<commit_message>
module 1 last updates all projects
</commit_message>
<xml_diff>
--- a/week-01/How did we do_  La Mesa (1-6).xlsx
+++ b/week-01/How did we do_  La Mesa (1-6).xlsx
@@ -1,21 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sthefanieramirez\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sthef\data-analytics\week-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC08DCA0-C15E-49C1-BADA-37B464DD814E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76FB59D9-821C-4957-A2C2-605BB95CF7E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-2340" yWindow="350" windowWidth="18450" windowHeight="10050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4620" yWindow="948" windowWidth="18492" windowHeight="10968" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="La_Mesa_Survey" sheetId="1" r:id="rId1"/>
+    <sheet name="Grapht" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="11" r:id="rId3"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="54">
   <si>
     <t>ID</t>
   </si>
@@ -189,6 +193,22 @@
   </si>
   <si>
     <t>Time to complete</t>
+  </si>
+  <si>
+    <t>Row Labels</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Sum of ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sum of How likely are you to visit us again?
+</t>
+  </si>
+  <si>
+    <t>(All)</t>
   </si>
 </sst>
 </file>
@@ -197,7 +217,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -228,13 +248,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -255,25 +275,48 @@
     <xf numFmtId="45" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
-    <dxf>
-      <numFmt numFmtId="28" formatCode="mm:ss"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="32">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm:ss"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -281,7 +324,68 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm:ss"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="28" formatCode="mm:ss"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm:ss"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -301,6 +405,10 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm:ss"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -312,15 +420,25 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="28" formatCode="mm:ss"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm:ss"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
@@ -336,27 +454,2390 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[How did we do_  La Mesa (1-6).xlsx]Grapht!PivotTable1</c:name>
+    <c:fmtId val="0"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="4"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="5"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="6"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="7"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="8"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="9"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="10"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="11"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="12"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="13"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="14"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="15"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="16"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="17"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="18"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="19"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="20"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="21"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="2.3718642976319409E-2"/>
+          <c:y val="0.1940233661268532"/>
+          <c:w val="0.77497227344723174"/>
+          <c:h val="0.51744752144077233"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Grapht!$B$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Sum of ID</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:multiLvlStrRef>
+              <c:f>Grapht!$A$5:$A$19</c:f>
+              <c:multiLvlStrCache>
+                <c:ptCount val="6"/>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>A loyalty number at checkout</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>A loyalty number at checkout</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>A mobile app</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>A mobile app</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>A mobile app</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>A mobile app</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>10-20 minutes</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>10-20 minutes</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>Over 30 minutes</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>Under 10 minutes</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>Under 10 minutes</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>A few times a month</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>Once or twice so far</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>This is my first time</c:v>
+                  </c:pt>
+                </c:lvl>
+              </c:multiLvlStrCache>
+            </c:multiLvlStrRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Grapht!$B$5:$B$19</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000005-1CA4-4108-8040-DAEA168C31AF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Grapht!$C$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Sum of How likely are you to visit us again?
+</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:multiLvlStrRef>
+              <c:f>Grapht!$A$5:$A$19</c:f>
+              <c:multiLvlStrCache>
+                <c:ptCount val="6"/>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>A loyalty number at checkout</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>A loyalty number at checkout</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>A mobile app</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>A mobile app</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>A mobile app</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>A mobile app</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>10-20 minutes</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>10-20 minutes</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>Over 30 minutes</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>Under 10 minutes</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>Under 10 minutes</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>A few times a month</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>Once or twice so far</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>This is my first time</c:v>
+                  </c:pt>
+                </c:lvl>
+              </c:multiLvlStrCache>
+            </c:multiLvlStrRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Grapht!$C$5:$C$19</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-1CA4-4108-8040-DAEA168C31AF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1952081599"/>
+        <c:axId val="1597407039"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1952081599"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1597407039"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1597407039"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1952081599"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{828A6150-9601-343C-6ED5-1B8FE7E2DBC9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="sthef" refreshedDate="46125.516952893522" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="6" xr:uid="{E4291998-D4A5-4C0F-81FB-05796B954221}">
+  <cacheSource type="worksheet">
+    <worksheetSource name="Table1"/>
+  </cacheSource>
+  <cacheFields count="15">
+    <cacheField name="ID" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="6" count="6">
+        <n v="1"/>
+        <n v="2"/>
+        <n v="3"/>
+        <n v="4"/>
+        <n v="5"/>
+        <n v="6"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Start time" numFmtId="165">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-04-10T01:04:12" maxDate="2026-04-10T13:46:45"/>
+    </cacheField>
+    <cacheField name="Completion time" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="46122.056770833296" maxValue="46122.574814814798"/>
+    </cacheField>
+    <cacheField name="Time to complete" numFmtId="45">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="1899-12-30T00:00:20" maxDate="1899-12-30T00:17:33"/>
+    </cacheField>
+    <cacheField name="Email" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Name" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Last modified time" numFmtId="164">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="How would you rate your overall experience today?_x000a_" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="2" maxValue="5"/>
+    </cacheField>
+    <cacheField name="How long did it take for your food to arrive after ordering?_x000a_" numFmtId="0">
+      <sharedItems count="3">
+        <s v="Under 10 minutes"/>
+        <s v="10-20 minutes"/>
+        <s v="Over 30 minutes"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="What stood out most about your visit today?_x000a_" numFmtId="0">
+      <sharedItems count="6">
+        <s v="Friendly service;"/>
+        <s v="Food quality &amp; flavor;Friendly service;Cleanliness;"/>
+        <s v="Food quality &amp; flavor;Friendly service;Speed of service;"/>
+        <s v="Food quality &amp; flavor;Restaurant atmosphere / vibe;"/>
+        <s v="Food quality &amp; flavor;Friendly service;Restaurant atmosphere / vibe;Cleanliness;"/>
+        <s v="Food quality &amp; flavor;Friendly service;Restaurant atmosphere / vibe;Cleanliness;Speed of service;"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="How often do you visit La Mesa Alegre?_x000a_" numFmtId="0">
+      <sharedItems count="3">
+        <s v="This is my first time"/>
+        <s v="Once or twice so far"/>
+        <s v="A few times a month"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="What kind of rewards would make you more likely to come back regularly?" numFmtId="0">
+      <sharedItems count="4">
+        <s v="Birthday reward;Free item after a set number of visits;"/>
+        <s v="Birthday reward;"/>
+        <s v="Free item after a set number of visits;Discount on a future order;"/>
+        <s v="Free item after a set number of visits;"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="How would you prefer to track your rewards?_x000a_" numFmtId="0">
+      <sharedItems count="2">
+        <s v="A mobile app"/>
+        <s v="A loyalty number at checkout"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="How likely are you to visit us again?_x000a_" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="3" maxValue="10" count="5">
+        <n v="10"/>
+        <n v="8"/>
+        <n v="7"/>
+        <n v="3"/>
+        <n v="9"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Is there anything else you'd like us to know something you loved, something we could improve, or any suggestions?" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="6">
+  <r>
+    <x v="0"/>
+    <d v="2026-04-10T01:04:12"/>
+    <n v="46122.056770833296"/>
+    <d v="1899-12-30T00:17:33"/>
+    <s v="nmiranda@my.yearupunited.org"/>
+    <s v="natalia miranda"/>
+    <m/>
+    <n v="5"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <m/>
+  </r>
+  <r>
+    <x v="1"/>
+    <d v="2026-04-10T09:57:17"/>
+    <n v="46122.415011574099"/>
+    <d v="1899-12-30T00:00:20"/>
+    <s v="dsanchez1@my.yearupunited.org"/>
+    <s v="dahlia sanchez"/>
+    <m/>
+    <n v="5"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="1"/>
+    <m/>
+  </r>
+  <r>
+    <x v="2"/>
+    <d v="2026-04-10T10:47:57"/>
+    <n v="46122.4528587963"/>
+    <d v="1899-12-30T00:04:10"/>
+    <s v="jgoode@my.yearupunited.org"/>
+    <s v="jeremiah goode"/>
+    <m/>
+    <n v="5"/>
+    <x v="1"/>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="1"/>
+    <x v="2"/>
+    <s v="I love coming here with family. The service is fast and friendly, and the restaurant is super clean. I would say maybe add a little more deals because the menu can be very expensive at times."/>
+  </r>
+  <r>
+    <x v="3"/>
+    <d v="2026-04-10T11:10:53"/>
+    <n v="46122.467777777798"/>
+    <d v="1899-12-30T00:02:43"/>
+    <s v="dlomeli@my.yearupunited.org"/>
+    <s v="destiney lomeli"/>
+    <m/>
+    <n v="2"/>
+    <x v="2"/>
+    <x v="3"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="3"/>
+    <s v="My food took longer than an hour to arrive and when I'd ask for updates I'd get ignored! Please improve your customer service."/>
+  </r>
+  <r>
+    <x v="4"/>
+    <d v="2026-04-10T11:54:45"/>
+    <n v="46122.497002314798"/>
+    <d v="1899-12-30T00:00:56"/>
+    <s v="BHambleton@YearUp.org"/>
+    <s v="Bess Hambleton"/>
+    <m/>
+    <m/>
+    <x v="1"/>
+    <x v="4"/>
+    <x v="1"/>
+    <x v="3"/>
+    <x v="1"/>
+    <x v="0"/>
+    <s v="more cushy seats"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <d v="2026-04-10T13:46:45"/>
+    <n v="46122.574814814798"/>
+    <d v="1899-12-30T00:00:59"/>
+    <s v="bcarrillo-valencia@my.yearupunited.org"/>
+    <s v="brandon carrillo-valencia"/>
+    <m/>
+    <n v="5"/>
+    <x v="1"/>
+    <x v="5"/>
+    <x v="1"/>
+    <x v="2"/>
+    <x v="0"/>
+    <x v="4"/>
+    <s v="Very good service!"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{52D429DF-E675-47D0-8CAB-11D1C339ED87}" name="PivotTable1" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+  <location ref="A4:C19" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="15">
+    <pivotField dataField="1" showAll="0">
+      <items count="7">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="165" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="45" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="1"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="2"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="5">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0">
+      <items count="6">
+        <item x="3"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="3">
+    <field x="10"/>
+    <field x="8"/>
+    <field x="12"/>
+  </rowFields>
+  <rowItems count="15">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="2">
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="2">
+      <x/>
+    </i>
+    <i r="2">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="2">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="2">
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="2">
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="11" hier="-1"/>
+  </pageFields>
+  <dataFields count="2">
+    <dataField name="Sum of ID" fld="0" baseField="0" baseItem="0"/>
+    <dataField name="Sum of How likely are you to visit us again?_x000a_" fld="13" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="6">
+    <chartFormat chart="0" format="10" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="14" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="15" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="8" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="16" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="8" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="17" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="8" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="18" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="8" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:O7" totalsRowShown="0" dataDxfId="5">
-  <autoFilter ref="A1:O7" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:O8" totalsRowCount="1" headerRowDxfId="30" dataDxfId="31">
+  <autoFilter ref="A1:O7" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Start time" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Completion time" dataDxfId="2"/>
-    <tableColumn id="15" xr3:uid="{718CF1A5-A920-4B79-9363-494CD09553A3}" name="Time to complete" dataDxfId="0">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" dataDxfId="29" totalsRowDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Start time" dataDxfId="28" totalsRowDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Completion time" dataDxfId="27" totalsRowDxfId="12"/>
+    <tableColumn id="15" xr3:uid="{718CF1A5-A920-4B79-9363-494CD09553A3}" name="Time to complete" totalsRowFunction="custom" dataDxfId="26" totalsRowDxfId="11">
       <calculatedColumnFormula>C2-B2</calculatedColumnFormula>
+      <totalsRowFormula>AVERAGE(Table1[Time to complete])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Last modified time" dataDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="How would you rate your overall experience today?_x000a_" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="How long did it take for your food to arrive after ordering?_x000a_" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="What stood out most about your visit today?_x000a_" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="How often do you visit La Mesa Alegre?_x000a_" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="What kind of rewards would make you more likely to come back regularly?" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="How would you prefer to track your rewards?_x000a_" dataDxfId="8"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="How likely are you to visit us again?_x000a_" dataDxfId="7"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Is there anything else you'd like us to know something you loved, something we could improve, or any suggestions?" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="25" totalsRowDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name" dataDxfId="24" totalsRowDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Last modified time" dataDxfId="23" totalsRowDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="How would you rate your overall experience today?_x000a_" totalsRowFunction="custom" dataDxfId="22" totalsRowDxfId="7">
+      <totalsRowFormula>AVERAGE(H2:H7)</totalsRowFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="How long did it take for your food to arrive after ordering?_x000a_" totalsRowFunction="custom" dataDxfId="21" totalsRowDxfId="6">
+      <totalsRowFormula>COUNTIF(I2:I7, "Under 10 minutes")</totalsRowFormula>
+    </tableColumn>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="What stood out most about your visit today?_x000a_" dataDxfId="20" totalsRowDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="How often do you visit La Mesa Alegre?_x000a_" totalsRowFunction="custom" dataDxfId="19" totalsRowDxfId="4">
+      <totalsRowFormula>COUNTIF(K2:K7, "Once or twice so far")</totalsRowFormula>
+    </tableColumn>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="What kind of rewards would make you more likely to come back regularly?" dataDxfId="18" totalsRowDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="How would you prefer to track your rewards?_x000a_" totalsRowFunction="custom" dataDxfId="15" totalsRowDxfId="2">
+      <totalsRowFormula>SUM(COUNTIF(Table1[How would you prefer to track your rewards?
+], "A mobile app"), COUNTIF(Table1[How would you prefer to track your rewards?
+], "A loyalty number at checkout"))</totalsRowFormula>
+    </tableColumn>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="How likely are you to visit us again?_x000a_" dataDxfId="17" totalsRowDxfId="1"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Is there anything else you'd like us to know something you loved, something we could improve, or any suggestions?" dataDxfId="16" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -659,63 +3140,65 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O7"/>
-  <sheetFormatPr defaultColWidth="18.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:O8"/>
+  <sheetFormatPr defaultColWidth="27.6640625" defaultRowHeight="67.8" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="18.6328125" style="2"/>
-    <col min="3" max="3" width="22" style="7" customWidth="1"/>
-    <col min="4" max="4" width="18.6328125" style="8"/>
-    <col min="15" max="15" width="52.26953125" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" style="2"/>
+    <col min="3" max="3" width="27.6640625" style="7"/>
+    <col min="4" max="4" width="27.6640625" style="8"/>
+    <col min="8" max="8" width="27.6640625" style="13"/>
+    <col min="10" max="10" width="27.6640625" style="1"/>
+    <col min="14" max="14" width="27.6640625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:15" s="15" customFormat="1" ht="67.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="1" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" s="1" customFormat="1" ht="67.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -726,7 +3209,7 @@
         <v>46122.056770833296</v>
       </c>
       <c r="D2" s="9">
-        <f t="shared" ref="D2:D7" si="0">C2-B2</f>
+        <f>C2-B2</f>
         <v>1.2187499996798579E-2</v>
       </c>
       <c r="E2" s="1" t="s">
@@ -736,7 +3219,7 @@
         <v>15</v>
       </c>
       <c r="G2" s="4"/>
-      <c r="H2" s="1">
+      <c r="H2" s="14">
         <v>5</v>
       </c>
       <c r="I2" s="1" t="s">
@@ -754,11 +3237,11 @@
       <c r="M2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="6">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:15" s="1" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" s="1" customFormat="1" ht="67.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -769,7 +3252,7 @@
         <v>46122.415011574099</v>
       </c>
       <c r="D3" s="9">
-        <f t="shared" si="0"/>
+        <f>C3-B3</f>
         <v>2.3148149921325967E-4</v>
       </c>
       <c r="E3" s="1" t="s">
@@ -779,7 +3262,7 @@
         <v>22</v>
       </c>
       <c r="G3" s="4"/>
-      <c r="H3" s="1">
+      <c r="H3" s="14">
         <v>5</v>
       </c>
       <c r="I3" s="1" t="s">
@@ -797,11 +3280,11 @@
       <c r="M3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="6">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:15" s="1" customFormat="1" ht="61.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" s="1" customFormat="1" ht="67.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6">
         <v>3</v>
       </c>
@@ -812,7 +3295,7 @@
         <v>46122.4528587963</v>
       </c>
       <c r="D4" s="9">
-        <f t="shared" si="0"/>
+        <f>C4-B4</f>
         <v>2.8935184964211658E-3</v>
       </c>
       <c r="E4" s="1" t="s">
@@ -822,7 +3305,7 @@
         <v>27</v>
       </c>
       <c r="G4" s="4"/>
-      <c r="H4" s="1">
+      <c r="H4" s="14">
         <v>5</v>
       </c>
       <c r="I4" s="1" t="s">
@@ -840,14 +3323,14 @@
       <c r="M4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="6">
         <v>7</v>
       </c>
       <c r="O4" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:15" s="1" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" s="1" customFormat="1" ht="67.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -858,7 +3341,7 @@
         <v>46122.467777777798</v>
       </c>
       <c r="D5" s="9">
-        <f t="shared" si="0"/>
+        <f>C5-B5</f>
         <v>1.8865741003537551E-3</v>
       </c>
       <c r="E5" s="1" t="s">
@@ -868,7 +3351,7 @@
         <v>35</v>
       </c>
       <c r="G5" s="4"/>
-      <c r="H5" s="1">
+      <c r="H5" s="14">
         <v>2</v>
       </c>
       <c r="I5" s="1" t="s">
@@ -886,14 +3369,14 @@
       <c r="M5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="6">
         <v>3</v>
       </c>
       <c r="O5" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:15" s="1" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" s="1" customFormat="1" ht="67.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -904,7 +3387,7 @@
         <v>46122.497002314798</v>
       </c>
       <c r="D6" s="9">
-        <f t="shared" si="0"/>
+        <f>C6-B6</f>
         <v>6.4814809593372047E-4</v>
       </c>
       <c r="E6" s="1" t="s">
@@ -914,6 +3397,7 @@
         <v>40</v>
       </c>
       <c r="G6" s="4"/>
+      <c r="H6" s="14"/>
       <c r="I6" s="1" t="s">
         <v>28</v>
       </c>
@@ -929,14 +3413,14 @@
       <c r="M6" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="6">
         <v>10</v>
       </c>
       <c r="O6" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:15" s="1" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" s="1" customFormat="1" ht="67.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -947,7 +3431,7 @@
         <v>46122.574814814798</v>
       </c>
       <c r="D7" s="9">
-        <f t="shared" si="0"/>
+        <f>C7-B7</f>
         <v>6.8287039903225377E-4</v>
       </c>
       <c r="E7" s="1" t="s">
@@ -957,7 +3441,7 @@
         <v>45</v>
       </c>
       <c r="G7" s="4"/>
-      <c r="H7" s="1">
+      <c r="H7" s="14">
         <v>5</v>
       </c>
       <c r="I7" s="1" t="s">
@@ -975,12 +3459,46 @@
       <c r="M7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="6">
         <v>9</v>
       </c>
       <c r="O7" s="1" t="s">
         <v>47</v>
       </c>
+    </row>
+    <row r="8" spans="1:15" ht="67.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="10"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="9">
+        <f>AVERAGE(Table1[Time to complete])</f>
+        <v>3.0883487646254557E-3</v>
+      </c>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="10">
+        <f>AVERAGE(H2:H7)</f>
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="I8" s="10">
+        <f>COUNTIF(I2:I7, "Under 10 minutes")</f>
+        <v>2</v>
+      </c>
+      <c r="J8" s="12"/>
+      <c r="K8" s="10">
+        <f>COUNTIF(K2:K7, "Once or twice so far")</f>
+        <v>4</v>
+      </c>
+      <c r="L8" s="12"/>
+      <c r="M8" s="10">
+        <f>SUM(COUNTIF(Table1[How would you prefer to track your rewards?
+], "A mobile app"), COUNTIF(Table1[How would you prefer to track your rewards?
+], "A loyalty number at checkout"))</f>
+        <v>6</v>
+      </c>
+      <c r="N8" s="10"/>
+      <c r="O8" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -989,4 +3507,210 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EA76287-99C7-47DA-A3F0-22CA60CE7865}">
+  <dimension ref="A2:C19"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="62.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="43.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="43.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="19">
+        <v>3</v>
+      </c>
+      <c r="C5" s="19">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="19">
+        <v>3</v>
+      </c>
+      <c r="C6" s="19">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="19">
+        <v>3</v>
+      </c>
+      <c r="C7" s="19">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="19">
+        <v>17</v>
+      </c>
+      <c r="C8" s="19">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="19">
+        <v>11</v>
+      </c>
+      <c r="C9" s="19">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="19">
+        <v>5</v>
+      </c>
+      <c r="C10" s="19">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="19">
+        <v>6</v>
+      </c>
+      <c r="C11" s="19">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="19">
+        <v>4</v>
+      </c>
+      <c r="C12" s="19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="19">
+        <v>4</v>
+      </c>
+      <c r="C13" s="19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="19">
+        <v>2</v>
+      </c>
+      <c r="C14" s="19">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="19">
+        <v>2</v>
+      </c>
+      <c r="C15" s="19">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="19">
+        <v>1</v>
+      </c>
+      <c r="C16" s="19">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="19">
+        <v>1</v>
+      </c>
+      <c r="C17" s="19">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="19">
+        <v>1</v>
+      </c>
+      <c r="C18" s="19">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" s="19">
+        <v>21</v>
+      </c>
+      <c r="C19" s="19">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>